<commit_message>
Restore the 2026-10-07 thermodynamic methanol chain for the freeze (revert of ba9db90 for code and data)
Brings back the model with recycled CO bounded by CO-hydrogenation equilibrium and the conversion cap, the candidate
builder, field pipeline, statistics, pruning, catalyst-cost and benchmark code of 86dcd76, the extraction records with
the unit-parsing fixes, and the Table 4 self-check reference for that model. Kept from main: the ammonia work after
86dcd76 (ED Fig. 7 code), the CI mode of the self-check gate, the verify mode of the statistics workflow. Manuscript,
captions, SI, SOURCE_OF_TRUTH and the text audit are not touched. Outputs still hold the 2026-10-07 primary (inlet
limit, 54/82) until the next commit switches the primary to step S5 on printed values.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/SourceData_EDFig1.xlsx
+++ b/source_data/SourceData_EDFig1.xlsx
@@ -714,13 +714,13 @@
         </is>
       </c>
       <c r="D7" t="n">
+        <v>130</v>
+      </c>
+      <c r="E7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F7" t="n">
         <v>129</v>
-      </c>
-      <c r="E7" t="n">
-        <v>129</v>
-      </c>
-      <c r="F7" t="n">
-        <v>128</v>
       </c>
       <c r="G7" t="n">
         <v>0.992</v>
@@ -746,13 +746,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E8" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F8" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G8" t="n">
         <v>0.961</v>
@@ -778,19 +778,19 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="E9" t="n">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="F9" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G9" t="n">
-        <v>0.959</v>
+        <v>0.922</v>
       </c>
       <c r="H9" t="n">
-        <v>0.975</v>
+        <v>0.945</v>
       </c>
     </row>
     <row r="10">
@@ -874,19 +874,19 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="E12" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F12" t="n">
         <v>15</v>
       </c>
       <c r="G12" t="n">
-        <v>0.112</v>
+        <v>0.113</v>
       </c>
       <c r="H12" t="n">
-        <v>0.313</v>
+        <v>0.323</v>
       </c>
     </row>
     <row r="13">
@@ -973,16 +973,16 @@
         <v>32</v>
       </c>
       <c r="E15" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="F15" t="n">
         <v>3</v>
       </c>
       <c r="G15" t="n">
-        <v>0.5</v>
+        <v>0.167</v>
       </c>
       <c r="H15" t="n">
-        <v>0.667</v>
+        <v>0.278</v>
       </c>
     </row>
   </sheetData>
@@ -1081,13 +1081,13 @@
         <v>547</v>
       </c>
       <c r="C4" t="n">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="D4" t="n">
-        <v>0.962</v>
+        <v>0.965</v>
       </c>
       <c r="E4" t="n">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="5">
@@ -1106,7 +1106,7 @@
         <v>0.985</v>
       </c>
       <c r="E5" t="n">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6">
@@ -1119,10 +1119,10 @@
         <v>741</v>
       </c>
       <c r="C6" t="n">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="D6" t="n">
-        <v>0.968</v>
+        <v>0.97</v>
       </c>
       <c r="E6" t="n">
         <v>647</v>

</xml_diff>